<commit_message>
Completed cleaning all the plaform SW files, each one now have 15 columns.
Next: Add a merging script and create a final output file
</commit_message>
<xml_diff>
--- a/SWTest/Outputs/Finalists/Nebula_Galaxy_Analysis_Final.xlsx
+++ b/SWTest/Outputs/Finalists/Nebula_Galaxy_Analysis_Final.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\Outputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\u245231\Quan_Vo\Local_Dev\complete-pandas-tutorial\SWTest\Outputs\Finalists\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BEEE9AE-2C2B-447C-BECC-8AC884786182}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E33651EA-21E3-4366-891C-6871762DFDF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2400" yWindow="3030" windowWidth="14190" windowHeight="8460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1787" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1626" uniqueCount="394">
   <si>
     <t>SPN</t>
   </si>
@@ -1259,18 +1259,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1583,8 +1577,8 @@
     <col min="6" max="6" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="59.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.28515625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="34.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="27.5703125" bestFit="1" customWidth="1"/>
@@ -1618,10 +1612,10 @@
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>10</v>
@@ -1662,13 +1656,11 @@
       <c r="H2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="3">
+      <c r="I2" s="2">
         <v>127</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
       <c r="L2" s="2" t="s">
         <v>19</v>
       </c>
@@ -1701,13 +1693,11 @@
       <c r="H3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="3">
+      <c r="I3" s="2">
         <v>127</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
       <c r="L3" s="2" t="s">
         <v>19</v>
       </c>
@@ -1740,15 +1730,13 @@
       <c r="H4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="2">
+        <v>127</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="J4" s="3">
-        <v>127</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K4" s="2"/>
       <c r="L4" s="2" t="s">
         <v>19</v>
       </c>
@@ -1782,14 +1770,12 @@
         <v>20</v>
       </c>
       <c r="I5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
         <v>19</v>
       </c>
@@ -1822,15 +1808,13 @@
       <c r="H6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="2">
+        <v>3</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="3">
-        <v>3</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K6" s="2"/>
       <c r="L6" s="2" t="s">
         <v>19</v>
       </c>
@@ -1863,15 +1847,13 @@
       <c r="H7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="2">
+        <v>3</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="3">
-        <v>3</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K7" s="2"/>
       <c r="L7" s="2" t="s">
         <v>19</v>
       </c>
@@ -1904,15 +1886,13 @@
       <c r="H8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="2">
+        <v>3</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J8" s="3">
-        <v>3</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
         <v>19</v>
       </c>
@@ -1945,15 +1925,13 @@
       <c r="H9" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="2">
+        <v>4</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="3">
-        <v>4</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K9" s="2"/>
       <c r="L9" s="2" t="s">
         <v>19</v>
       </c>
@@ -1986,15 +1964,13 @@
       <c r="H10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="2">
+        <v>4</v>
+      </c>
+      <c r="J10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J10" s="3">
-        <v>4</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
         <v>19</v>
       </c>
@@ -2027,15 +2003,13 @@
       <c r="H11" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="2">
+        <v>4</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J11" s="3">
-        <v>4</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
         <v>19</v>
       </c>
@@ -2069,14 +2043,12 @@
         <v>20</v>
       </c>
       <c r="I12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J12" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
         <v>19</v>
       </c>
@@ -2110,14 +2082,12 @@
         <v>20</v>
       </c>
       <c r="I13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J13" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J13" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K13" s="2"/>
       <c r="L13" s="2" t="s">
         <v>19</v>
       </c>
@@ -2151,14 +2121,12 @@
         <v>20</v>
       </c>
       <c r="I14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="J14" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K14" s="2"/>
       <c r="L14" s="2" t="s">
         <v>19</v>
       </c>
@@ -2191,15 +2159,13 @@
       <c r="H15" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="I15" s="2">
+        <v>206</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J15" s="3">
-        <v>206</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K15" s="2"/>
       <c r="L15" s="2" t="s">
         <v>19</v>
       </c>
@@ -2235,14 +2201,12 @@
         <v>37</v>
       </c>
       <c r="I16" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="J16" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K16" s="2"/>
       <c r="L16" s="2" t="s">
         <v>19</v>
       </c>
@@ -2275,13 +2239,11 @@
       <c r="H17" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="3">
+      <c r="I17" s="2">
         <v>202</v>
       </c>
-      <c r="K17" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
       <c r="L17" s="2" t="s">
         <v>19</v>
       </c>
@@ -2314,13 +2276,11 @@
       <c r="H18" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I18" s="2"/>
-      <c r="J18" s="3">
+      <c r="I18" s="2">
         <v>67</v>
       </c>
-      <c r="K18" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
       <c r="L18" s="2" t="s">
         <v>19</v>
       </c>
@@ -2353,13 +2313,11 @@
       <c r="H19" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I19" s="2"/>
-      <c r="J19" s="3">
+      <c r="I19" s="2">
         <v>67</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
       <c r="L19" s="2" t="s">
         <v>19</v>
       </c>
@@ -2392,13 +2350,11 @@
       <c r="H20" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I20" s="2"/>
-      <c r="J20" s="3">
+      <c r="I20" s="2">
         <v>67</v>
       </c>
-      <c r="K20" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
       <c r="L20" s="2" t="s">
         <v>19</v>
       </c>
@@ -2431,13 +2387,11 @@
       <c r="H21" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I21" s="2"/>
-      <c r="J21" s="3">
+      <c r="I21" s="2">
         <v>67</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
       <c r="L21" s="2" t="s">
         <v>19</v>
       </c>
@@ -2470,13 +2424,11 @@
       <c r="H22" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I22" s="2"/>
-      <c r="J22" s="3" t="s">
+      <c r="I22" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K22" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J22" s="2"/>
+      <c r="K22" s="2"/>
       <c r="L22" s="2" t="s">
         <v>19</v>
       </c>
@@ -2511,13 +2463,11 @@
       <c r="H23" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I23" s="2"/>
-      <c r="J23" s="3" t="s">
+      <c r="I23" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K23" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
       <c r="L23" s="2" t="s">
         <v>19</v>
       </c>
@@ -2550,13 +2500,11 @@
       <c r="H24" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I24" s="2"/>
-      <c r="J24" s="3">
+      <c r="I24" s="2">
         <v>45</v>
       </c>
-      <c r="K24" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
       <c r="L24" s="2" t="s">
         <v>19</v>
       </c>
@@ -2589,13 +2537,11 @@
       <c r="H25" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I25" s="2"/>
-      <c r="J25" s="3">
+      <c r="I25" s="2">
         <v>45</v>
       </c>
-      <c r="K25" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J25" s="2"/>
+      <c r="K25" s="2"/>
       <c r="L25" s="2" t="s">
         <v>19</v>
       </c>
@@ -2628,13 +2574,11 @@
       <c r="H26" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I26" s="2"/>
-      <c r="J26" s="3" t="s">
+      <c r="I26" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J26" s="2"/>
+      <c r="K26" s="2"/>
       <c r="L26" s="2" t="s">
         <v>19</v>
       </c>
@@ -2667,13 +2611,11 @@
       <c r="H27" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I27" s="2"/>
-      <c r="J27" s="3" t="s">
+      <c r="I27" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="K27" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
       <c r="L27" s="2" t="s">
         <v>19</v>
       </c>
@@ -2706,13 +2648,11 @@
       <c r="H28" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I28" s="2"/>
-      <c r="J28" s="3">
+      <c r="I28" s="2">
         <v>121</v>
       </c>
-      <c r="K28" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J28" s="2"/>
+      <c r="K28" s="2"/>
       <c r="L28" s="2" t="s">
         <v>19</v>
       </c>
@@ -2747,13 +2687,11 @@
       <c r="H29" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I29" s="2"/>
-      <c r="J29" s="3">
+      <c r="I29" s="2">
         <v>121</v>
       </c>
-      <c r="K29" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J29" s="2"/>
+      <c r="K29" s="2"/>
       <c r="L29" s="2" t="s">
         <v>19</v>
       </c>
@@ -2787,14 +2725,12 @@
         <v>37</v>
       </c>
       <c r="I30" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="J30" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="J30" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="K30" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K30" s="2"/>
       <c r="L30" s="2" t="s">
         <v>19</v>
       </c>
@@ -2829,10 +2765,10 @@
       <c r="H31" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I31" s="2"/>
-      <c r="J31" s="3">
+      <c r="I31" s="2">
         <v>108</v>
       </c>
+      <c r="J31" s="2"/>
       <c r="K31" s="2" t="s">
         <v>18</v>
       </c>
@@ -2872,10 +2808,10 @@
       <c r="H32" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I32" s="2"/>
-      <c r="J32" s="3">
+      <c r="I32" s="2">
         <v>108</v>
       </c>
+      <c r="J32" s="2"/>
       <c r="K32" s="2" t="s">
         <v>18</v>
       </c>
@@ -2915,10 +2851,10 @@
       <c r="H33" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="I33" s="2"/>
-      <c r="J33" s="3">
+      <c r="I33" s="2">
         <v>108</v>
       </c>
+      <c r="J33" s="2"/>
       <c r="K33" s="2" t="s">
         <v>18</v>
       </c>
@@ -2957,14 +2893,12 @@
         <v>37</v>
       </c>
       <c r="I34" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J34" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J34" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="K34" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K34" s="2"/>
       <c r="L34" s="2" t="s">
         <v>19</v>
       </c>
@@ -2997,15 +2931,13 @@
       <c r="H35" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I35" s="2" t="s">
+      <c r="I35" s="2">
+        <v>88</v>
+      </c>
+      <c r="J35" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J35" s="3">
-        <v>88</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K35" s="2"/>
       <c r="L35" s="2" t="s">
         <v>19</v>
       </c>
@@ -3039,14 +2971,12 @@
         <v>37</v>
       </c>
       <c r="I36" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="J36" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J36" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K36" s="2"/>
       <c r="L36" s="2" t="s">
         <v>19</v>
       </c>
@@ -3079,13 +3009,11 @@
       <c r="H37" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I37" s="2"/>
-      <c r="J37" s="3">
+      <c r="I37" s="2">
         <v>267</v>
       </c>
-      <c r="K37" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
       <c r="L37" s="2" t="s">
         <v>19</v>
       </c>
@@ -3118,13 +3046,11 @@
       <c r="H38" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I38" s="2"/>
-      <c r="J38" s="3" t="s">
+      <c r="I38" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="K38" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
       <c r="L38" s="2" t="s">
         <v>19</v>
       </c>
@@ -3159,13 +3085,11 @@
       <c r="H39" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I39" s="2"/>
-      <c r="J39" s="3">
+      <c r="I39" s="2">
         <v>268</v>
       </c>
-      <c r="K39" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
       <c r="L39" s="2" t="s">
         <v>19</v>
       </c>
@@ -3200,13 +3124,11 @@
       <c r="H40" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I40" s="2"/>
-      <c r="J40" s="3">
+      <c r="I40" s="2">
         <v>268</v>
       </c>
-      <c r="K40" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
       <c r="L40" s="2" t="s">
         <v>19</v>
       </c>
@@ -3239,15 +3161,13 @@
       <c r="H41" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I41" s="2" t="s">
+      <c r="I41" s="2">
+        <v>534</v>
+      </c>
+      <c r="J41" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J41" s="3">
-        <v>534</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K41" s="2"/>
       <c r="L41" s="2" t="s">
         <v>19</v>
       </c>
@@ -3280,13 +3200,11 @@
       <c r="H42" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I42" s="2"/>
-      <c r="J42" s="3">
+      <c r="I42" s="2">
         <v>112</v>
       </c>
-      <c r="K42" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J42" s="2"/>
+      <c r="K42" s="2"/>
       <c r="L42" s="2" t="s">
         <v>19</v>
       </c>
@@ -3319,13 +3237,11 @@
       <c r="H43" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I43" s="2"/>
-      <c r="J43" s="3">
+      <c r="I43" s="2">
         <v>112</v>
       </c>
-      <c r="K43" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J43" s="2"/>
+      <c r="K43" s="2"/>
       <c r="L43" s="2" t="s">
         <v>19</v>
       </c>
@@ -3358,13 +3274,11 @@
       <c r="H44" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I44" s="2"/>
-      <c r="J44" s="3">
+      <c r="I44" s="2">
         <v>267</v>
       </c>
-      <c r="K44" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J44" s="2"/>
+      <c r="K44" s="2"/>
       <c r="L44" s="2" t="s">
         <v>19</v>
       </c>
@@ -3399,13 +3313,11 @@
       <c r="H45" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I45" s="2"/>
-      <c r="J45" s="3" t="s">
+      <c r="I45" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="K45" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J45" s="2"/>
+      <c r="K45" s="2"/>
       <c r="L45" s="2" t="s">
         <v>19</v>
       </c>
@@ -3441,10 +3353,8 @@
         <v>37</v>
       </c>
       <c r="I46" s="2"/>
-      <c r="J46" s="3"/>
-      <c r="K46" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J46" s="2"/>
+      <c r="K46" s="2"/>
       <c r="L46" s="2" t="s">
         <v>19</v>
       </c>
@@ -3478,10 +3388,8 @@
         <v>37</v>
       </c>
       <c r="I47" s="2"/>
-      <c r="J47" s="3"/>
-      <c r="K47" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J47" s="2"/>
+      <c r="K47" s="2"/>
       <c r="L47" s="2" t="s">
         <v>19</v>
       </c>
@@ -3514,15 +3422,13 @@
       <c r="H48" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I48" s="2" t="s">
+      <c r="I48" s="2">
+        <v>590</v>
+      </c>
+      <c r="J48" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J48" s="3">
-        <v>590</v>
-      </c>
-      <c r="K48" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K48" s="2"/>
       <c r="L48" s="2" t="s">
         <v>19</v>
       </c>
@@ -3555,15 +3461,13 @@
       <c r="H49" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I49" s="2" t="s">
+      <c r="I49" s="2">
+        <v>112</v>
+      </c>
+      <c r="J49" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J49" s="3">
-        <v>112</v>
-      </c>
-      <c r="K49" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K49" s="2"/>
       <c r="L49" s="2" t="s">
         <v>19</v>
       </c>
@@ -3596,13 +3500,11 @@
       <c r="H50" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I50" s="2"/>
-      <c r="J50" s="3">
+      <c r="I50" s="2">
         <v>112</v>
       </c>
-      <c r="K50" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J50" s="2"/>
+      <c r="K50" s="2"/>
       <c r="L50" s="2" t="s">
         <v>19</v>
       </c>
@@ -3637,13 +3539,11 @@
       <c r="H51" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I51" s="2"/>
-      <c r="J51" s="3" t="s">
+      <c r="I51" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="K51" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
       <c r="L51" s="2" t="s">
         <v>19</v>
       </c>
@@ -3676,13 +3576,11 @@
       <c r="H52" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I52" s="2"/>
-      <c r="J52" s="3">
+      <c r="I52" s="2">
         <v>874</v>
       </c>
-      <c r="K52" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J52" s="2"/>
+      <c r="K52" s="2"/>
       <c r="L52" s="2" t="s">
         <v>19</v>
       </c>
@@ -3717,13 +3615,11 @@
       <c r="H53" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I53" s="2" t="s">
+      <c r="I53" s="2"/>
+      <c r="J53" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J53" s="3"/>
-      <c r="K53" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K53" s="2"/>
       <c r="L53" s="2" t="s">
         <v>19</v>
       </c>
@@ -3759,10 +3655,8 @@
         <v>37</v>
       </c>
       <c r="I54" s="2"/>
-      <c r="J54" s="3"/>
-      <c r="K54" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J54" s="2"/>
+      <c r="K54" s="2"/>
       <c r="L54" s="2" t="s">
         <v>19</v>
       </c>
@@ -3797,15 +3691,13 @@
       <c r="H55" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I55" s="2" t="s">
+      <c r="I55" s="2">
+        <v>867</v>
+      </c>
+      <c r="J55" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J55" s="3">
-        <v>867</v>
-      </c>
-      <c r="K55" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K55" s="2"/>
       <c r="L55" s="2" t="s">
         <v>19</v>
       </c>
@@ -3839,10 +3731,8 @@
         <v>37</v>
       </c>
       <c r="I56" s="2"/>
-      <c r="J56" s="3"/>
-      <c r="K56" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J56" s="2"/>
+      <c r="K56" s="2"/>
       <c r="L56" s="2" t="s">
         <v>19</v>
       </c>
@@ -3878,14 +3768,12 @@
         <v>37</v>
       </c>
       <c r="I57" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="J57" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J57" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="K57" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K57" s="2"/>
       <c r="L57" s="2" t="s">
         <v>19</v>
       </c>
@@ -3920,15 +3808,13 @@
       <c r="H58" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I58" s="2" t="s">
+      <c r="I58" s="2">
+        <v>868</v>
+      </c>
+      <c r="J58" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="J58" s="3">
-        <v>868</v>
-      </c>
-      <c r="K58" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K58" s="2"/>
       <c r="L58" s="2" t="s">
         <v>19</v>
       </c>
@@ -3962,10 +3848,8 @@
         <v>37</v>
       </c>
       <c r="I59" s="2"/>
-      <c r="J59" s="3"/>
-      <c r="K59" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J59" s="2"/>
+      <c r="K59" s="2"/>
       <c r="L59" s="2" t="s">
         <v>19</v>
       </c>
@@ -4000,13 +3884,11 @@
       <c r="H60" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I60" s="2"/>
-      <c r="J60" s="3">
+      <c r="I60" s="2">
         <v>871</v>
       </c>
-      <c r="K60" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J60" s="2"/>
+      <c r="K60" s="2"/>
       <c r="L60" s="2" t="s">
         <v>19</v>
       </c>
@@ -4042,10 +3924,8 @@
         <v>37</v>
       </c>
       <c r="I61" s="2"/>
-      <c r="J61" s="3"/>
-      <c r="K61" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
       <c r="L61" s="2" t="s">
         <v>19</v>
       </c>
@@ -4079,14 +3959,12 @@
         <v>37</v>
       </c>
       <c r="I62" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="J62" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J62" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="K62" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K62" s="2"/>
       <c r="L62" s="2" t="s">
         <v>19</v>
       </c>
@@ -4121,13 +3999,11 @@
       <c r="H63" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I63" s="2" t="s">
+      <c r="I63" s="2"/>
+      <c r="J63" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J63" s="3"/>
-      <c r="K63" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K63" s="2"/>
       <c r="L63" s="2" t="s">
         <v>19</v>
       </c>
@@ -4163,10 +4039,8 @@
         <v>37</v>
       </c>
       <c r="I64" s="2"/>
-      <c r="J64" s="3"/>
-      <c r="K64" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J64" s="2"/>
+      <c r="K64" s="2"/>
       <c r="L64" s="2" t="s">
         <v>19</v>
       </c>
@@ -4199,13 +4073,11 @@
       <c r="H65" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I65" s="2" t="s">
+      <c r="I65" s="2"/>
+      <c r="J65" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J65" s="3"/>
-      <c r="K65" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K65" s="2"/>
       <c r="L65" s="2" t="s">
         <v>19</v>
       </c>
@@ -4238,13 +4110,11 @@
       <c r="H66" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I66" s="2"/>
-      <c r="J66" s="3" t="s">
+      <c r="I66" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="K66" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
       <c r="L66" s="2" t="s">
         <v>19</v>
       </c>
@@ -4279,15 +4149,13 @@
       <c r="H67" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I67" s="2" t="s">
+      <c r="I67" s="2">
+        <v>861</v>
+      </c>
+      <c r="J67" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="J67" s="3">
-        <v>861</v>
-      </c>
-      <c r="K67" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K67" s="2"/>
       <c r="L67" s="2" t="s">
         <v>19</v>
       </c>
@@ -4322,13 +4190,11 @@
       <c r="H68" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I68" s="2"/>
-      <c r="J68" s="3">
+      <c r="I68" s="2">
         <v>861</v>
       </c>
-      <c r="K68" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J68" s="2"/>
+      <c r="K68" s="2"/>
       <c r="L68" s="2" t="s">
         <v>19</v>
       </c>
@@ -4361,13 +4227,11 @@
       <c r="H69" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I69" s="2"/>
-      <c r="J69" s="3">
+      <c r="I69" s="2">
         <v>861</v>
       </c>
-      <c r="K69" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J69" s="2"/>
+      <c r="K69" s="2"/>
       <c r="L69" s="2" t="s">
         <v>19</v>
       </c>
@@ -4402,13 +4266,11 @@
       <c r="H70" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I70" s="2"/>
-      <c r="J70" s="3">
+      <c r="I70" s="2">
         <v>861</v>
       </c>
-      <c r="K70" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J70" s="2"/>
+      <c r="K70" s="2"/>
       <c r="L70" s="2" t="s">
         <v>19</v>
       </c>
@@ -4441,13 +4303,11 @@
       <c r="H71" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I71" s="2"/>
-      <c r="J71" s="3">
+      <c r="I71" s="2">
         <v>861</v>
       </c>
-      <c r="K71" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J71" s="2"/>
+      <c r="K71" s="2"/>
       <c r="L71" s="2" t="s">
         <v>19</v>
       </c>
@@ -4480,13 +4340,11 @@
       <c r="H72" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I72" s="2"/>
-      <c r="J72" s="3" t="s">
+      <c r="I72" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="K72" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J72" s="2"/>
+      <c r="K72" s="2"/>
       <c r="L72" s="2" t="s">
         <v>19</v>
       </c>
@@ -4519,13 +4377,11 @@
       <c r="H73" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I73" s="2"/>
-      <c r="J73" s="3" t="s">
+      <c r="I73" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="K73" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
       <c r="L73" s="2" t="s">
         <v>19</v>
       </c>
@@ -4560,13 +4416,11 @@
       <c r="H74" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I74" s="2"/>
-      <c r="J74" s="3" t="s">
+      <c r="I74" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="K74" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J74" s="2"/>
+      <c r="K74" s="2"/>
       <c r="L74" s="2" t="s">
         <v>19</v>
       </c>
@@ -4599,15 +4453,13 @@
       <c r="H75" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I75" s="2" t="s">
+      <c r="I75" s="2">
+        <v>61</v>
+      </c>
+      <c r="J75" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="J75" s="3">
-        <v>61</v>
-      </c>
-      <c r="K75" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K75" s="2"/>
       <c r="L75" s="2" t="s">
         <v>19</v>
       </c>
@@ -4640,13 +4492,11 @@
       <c r="H76" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I76" s="2"/>
-      <c r="J76" s="3">
+      <c r="I76" s="2">
         <v>869</v>
       </c>
-      <c r="K76" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J76" s="2"/>
+      <c r="K76" s="2"/>
       <c r="L76" s="2" t="s">
         <v>19</v>
       </c>
@@ -4679,13 +4529,11 @@
       <c r="H77" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I77" s="2"/>
-      <c r="J77" s="3">
+      <c r="I77" s="2">
         <v>869</v>
       </c>
-      <c r="K77" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J77" s="2"/>
+      <c r="K77" s="2"/>
       <c r="L77" s="2" t="s">
         <v>19</v>
       </c>
@@ -4718,13 +4566,11 @@
       <c r="H78" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I78" s="2"/>
-      <c r="J78" s="3" t="s">
+      <c r="I78" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="K78" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J78" s="2"/>
+      <c r="K78" s="2"/>
       <c r="L78" s="2" t="s">
         <v>19</v>
       </c>
@@ -4757,13 +4603,11 @@
       <c r="H79" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I79" s="2"/>
-      <c r="J79" s="3">
+      <c r="I79" s="2">
         <v>869</v>
       </c>
-      <c r="K79" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J79" s="2"/>
+      <c r="K79" s="2"/>
       <c r="L79" s="2" t="s">
         <v>19</v>
       </c>
@@ -4796,13 +4640,11 @@
       <c r="H80" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I80" s="2"/>
-      <c r="J80" s="3">
+      <c r="I80" s="2">
         <v>869</v>
       </c>
-      <c r="K80" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J80" s="2"/>
+      <c r="K80" s="2"/>
       <c r="L80" s="2" t="s">
         <v>19</v>
       </c>
@@ -4835,13 +4677,11 @@
       <c r="H81" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I81" s="2"/>
-      <c r="J81" s="3">
+      <c r="I81" s="2">
         <v>869</v>
       </c>
-      <c r="K81" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J81" s="2"/>
+      <c r="K81" s="2"/>
       <c r="L81" s="2" t="s">
         <v>19</v>
       </c>
@@ -4874,13 +4714,11 @@
       <c r="H82" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I82" s="2"/>
-      <c r="J82" s="3">
+      <c r="I82" s="2">
         <v>61</v>
       </c>
-      <c r="K82" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J82" s="2"/>
+      <c r="K82" s="2"/>
       <c r="L82" s="2" t="s">
         <v>19</v>
       </c>
@@ -4914,10 +4752,8 @@
         <v>37</v>
       </c>
       <c r="I83" s="2"/>
-      <c r="J83" s="3"/>
-      <c r="K83" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J83" s="2"/>
+      <c r="K83" s="2"/>
       <c r="L83" s="2" t="s">
         <v>19</v>
       </c>
@@ -4951,10 +4787,8 @@
         <v>37</v>
       </c>
       <c r="I84" s="2"/>
-      <c r="J84" s="3"/>
-      <c r="K84" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J84" s="2"/>
+      <c r="K84" s="2"/>
       <c r="L84" s="2" t="s">
         <v>19</v>
       </c>
@@ -4987,13 +4821,11 @@
       <c r="H85" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I85" s="2"/>
-      <c r="J85" s="3" t="s">
+      <c r="I85" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K85" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J85" s="2"/>
+      <c r="K85" s="2"/>
       <c r="L85" s="2" t="s">
         <v>19</v>
       </c>
@@ -5026,13 +4858,11 @@
       <c r="H86" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I86" s="2"/>
-      <c r="J86" s="3" t="s">
+      <c r="I86" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="K86" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J86" s="2"/>
+      <c r="K86" s="2"/>
       <c r="L86" s="2" t="s">
         <v>19</v>
       </c>
@@ -5065,15 +4895,13 @@
       <c r="H87" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I87" s="2" t="s">
+      <c r="I87" s="2">
+        <v>265</v>
+      </c>
+      <c r="J87" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="J87" s="3">
-        <v>265</v>
-      </c>
-      <c r="K87" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K87" s="2"/>
       <c r="L87" s="2" t="s">
         <v>19</v>
       </c>
@@ -5106,13 +4934,11 @@
       <c r="H88" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I88" s="2"/>
-      <c r="J88" s="3" t="s">
+      <c r="I88" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="K88" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J88" s="2"/>
+      <c r="K88" s="2"/>
       <c r="L88" s="2" t="s">
         <v>19</v>
       </c>
@@ -5147,13 +4973,11 @@
       <c r="H89" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I89" s="2"/>
-      <c r="J89" s="3" t="s">
+      <c r="I89" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="K89" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J89" s="2"/>
+      <c r="K89" s="2"/>
       <c r="L89" s="2" t="s">
         <v>19</v>
       </c>
@@ -5188,13 +5012,11 @@
       <c r="H90" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I90" s="2"/>
-      <c r="J90" s="3">
+      <c r="I90" s="2">
         <v>579</v>
       </c>
-      <c r="K90" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J90" s="2"/>
+      <c r="K90" s="2"/>
       <c r="L90" s="2" t="s">
         <v>19</v>
       </c>
@@ -5227,13 +5049,11 @@
       <c r="H91" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I91" s="2"/>
-      <c r="J91" s="3">
+      <c r="I91" s="2">
         <v>579</v>
       </c>
-      <c r="K91" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J91" s="2"/>
+      <c r="K91" s="2"/>
       <c r="L91" s="2" t="s">
         <v>19</v>
       </c>
@@ -5266,13 +5086,11 @@
       <c r="H92" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I92" s="2"/>
-      <c r="J92" s="3" t="s">
+      <c r="I92" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="K92" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J92" s="2"/>
+      <c r="K92" s="2"/>
       <c r="L92" s="2" t="s">
         <v>19</v>
       </c>
@@ -5308,14 +5126,12 @@
         <v>37</v>
       </c>
       <c r="I93" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="J93" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J93" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="K93" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K93" s="2"/>
       <c r="L93" s="2" t="s">
         <v>19</v>
       </c>
@@ -5350,15 +5166,13 @@
       <c r="H94" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I94" s="2" t="s">
+      <c r="I94" s="2">
+        <v>579</v>
+      </c>
+      <c r="J94" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J94" s="3">
-        <v>579</v>
-      </c>
-      <c r="K94" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K94" s="2"/>
       <c r="L94" s="2" t="s">
         <v>19</v>
       </c>
@@ -5394,14 +5208,12 @@
         <v>37</v>
       </c>
       <c r="I95" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="J95" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="J95" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="K95" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K95" s="2"/>
       <c r="L95" s="2" t="s">
         <v>19</v>
       </c>
@@ -5436,13 +5248,11 @@
       <c r="H96" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I96" s="2"/>
-      <c r="J96" s="3">
+      <c r="I96" s="2">
         <v>265</v>
       </c>
-      <c r="K96" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J96" s="2"/>
+      <c r="K96" s="2"/>
       <c r="L96" s="2" t="s">
         <v>19</v>
       </c>
@@ -5477,13 +5287,11 @@
       <c r="H97" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I97" s="2"/>
-      <c r="J97" s="3">
+      <c r="I97" s="2">
         <v>265</v>
       </c>
-      <c r="K97" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J97" s="2"/>
+      <c r="K97" s="2"/>
       <c r="L97" s="2" t="s">
         <v>19</v>
       </c>
@@ -5517,14 +5325,12 @@
         <v>37</v>
       </c>
       <c r="I98" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="J98" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J98" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="K98" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K98" s="2"/>
       <c r="L98" s="2" t="s">
         <v>19</v>
       </c>
@@ -5559,13 +5365,11 @@
       <c r="H99" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I99" s="2"/>
-      <c r="J99" s="3" t="s">
+      <c r="I99" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="K99" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J99" s="2"/>
+      <c r="K99" s="2"/>
       <c r="L99" s="2" t="s">
         <v>19</v>
       </c>
@@ -5601,14 +5405,12 @@
         <v>37</v>
       </c>
       <c r="I100" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="J100" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="J100" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="K100" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K100" s="2"/>
       <c r="L100" s="2" t="s">
         <v>19</v>
       </c>
@@ -5643,13 +5445,11 @@
       <c r="H101" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I101" s="2"/>
-      <c r="J101" s="3" t="s">
+      <c r="I101" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K101" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J101" s="2"/>
+      <c r="K101" s="2"/>
       <c r="L101" s="2" t="s">
         <v>19</v>
       </c>
@@ -5684,13 +5484,11 @@
       <c r="H102" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I102" s="2"/>
-      <c r="J102" s="3" t="s">
+      <c r="I102" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K102" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J102" s="2"/>
+      <c r="K102" s="2"/>
       <c r="L102" s="2" t="s">
         <v>19</v>
       </c>
@@ -5725,13 +5523,11 @@
       <c r="H103" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I103" s="2"/>
-      <c r="J103" s="3" t="s">
+      <c r="I103" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K103" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J103" s="2"/>
+      <c r="K103" s="2"/>
       <c r="L103" s="2" t="s">
         <v>19</v>
       </c>
@@ -5766,13 +5562,11 @@
       <c r="H104" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I104" s="2"/>
-      <c r="J104" s="3" t="s">
+      <c r="I104" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K104" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J104" s="2"/>
+      <c r="K104" s="2"/>
       <c r="L104" s="2" t="s">
         <v>19</v>
       </c>
@@ -5805,13 +5599,11 @@
       <c r="H105" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I105" s="2"/>
-      <c r="J105" s="3" t="s">
+      <c r="I105" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K105" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J105" s="2"/>
+      <c r="K105" s="2"/>
       <c r="L105" s="2" t="s">
         <v>19</v>
       </c>
@@ -5847,10 +5639,8 @@
         <v>37</v>
       </c>
       <c r="I106" s="2"/>
-      <c r="J106" s="3"/>
-      <c r="K106" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J106" s="2"/>
+      <c r="K106" s="2"/>
       <c r="L106" s="2" t="s">
         <v>19</v>
       </c>
@@ -5885,13 +5675,11 @@
       <c r="H107" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I107" s="2"/>
-      <c r="J107" s="3" t="s">
+      <c r="I107" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="K107" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J107" s="2"/>
+      <c r="K107" s="2"/>
       <c r="L107" s="2" t="s">
         <v>19</v>
       </c>
@@ -5926,13 +5714,11 @@
       <c r="H108" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I108" s="2"/>
-      <c r="J108" s="3">
+      <c r="I108" s="2">
         <v>265</v>
       </c>
-      <c r="K108" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J108" s="2"/>
+      <c r="K108" s="2"/>
       <c r="L108" s="2" t="s">
         <v>19</v>
       </c>
@@ -5967,15 +5753,13 @@
       <c r="H109" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I109" s="2" t="s">
+      <c r="I109" s="2">
+        <v>265</v>
+      </c>
+      <c r="J109" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="J109" s="3">
-        <v>265</v>
-      </c>
-      <c r="K109" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K109" s="2"/>
       <c r="L109" s="2" t="s">
         <v>19</v>
       </c>
@@ -6010,13 +5794,11 @@
       <c r="H110" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I110" s="2"/>
-      <c r="J110" s="3">
+      <c r="I110" s="2">
         <v>265</v>
       </c>
-      <c r="K110" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J110" s="2"/>
+      <c r="K110" s="2"/>
       <c r="L110" s="2" t="s">
         <v>19</v>
       </c>
@@ -6049,13 +5831,11 @@
       <c r="H111" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I111" s="2"/>
-      <c r="J111" s="3">
+      <c r="I111" s="2">
         <v>265</v>
       </c>
-      <c r="K111" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J111" s="2"/>
+      <c r="K111" s="2"/>
       <c r="L111" s="2" t="s">
         <v>19</v>
       </c>
@@ -6089,10 +5869,8 @@
         <v>37</v>
       </c>
       <c r="I112" s="2"/>
-      <c r="J112" s="3"/>
-      <c r="K112" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J112" s="2"/>
+      <c r="K112" s="2"/>
       <c r="L112" s="2" t="s">
         <v>19</v>
       </c>
@@ -6126,10 +5904,8 @@
         <v>37</v>
       </c>
       <c r="I113" s="2"/>
-      <c r="J113" s="3"/>
-      <c r="K113" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J113" s="2"/>
+      <c r="K113" s="2"/>
       <c r="L113" s="2" t="s">
         <v>19</v>
       </c>
@@ -6163,10 +5939,8 @@
         <v>37</v>
       </c>
       <c r="I114" s="2"/>
-      <c r="J114" s="3"/>
-      <c r="K114" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J114" s="2"/>
+      <c r="K114" s="2"/>
       <c r="L114" s="2" t="s">
         <v>19</v>
       </c>
@@ -6200,10 +5974,8 @@
         <v>37</v>
       </c>
       <c r="I115" s="2"/>
-      <c r="J115" s="3"/>
-      <c r="K115" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J115" s="2"/>
+      <c r="K115" s="2"/>
       <c r="L115" s="2" t="s">
         <v>19</v>
       </c>
@@ -6237,10 +6009,8 @@
         <v>37</v>
       </c>
       <c r="I116" s="2"/>
-      <c r="J116" s="3"/>
-      <c r="K116" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J116" s="2"/>
+      <c r="K116" s="2"/>
       <c r="L116" s="2" t="s">
         <v>19</v>
       </c>
@@ -6275,13 +6045,11 @@
       <c r="H117" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I117" s="2"/>
-      <c r="J117" s="3">
+      <c r="I117" s="2">
         <v>317</v>
       </c>
-      <c r="K117" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J117" s="2"/>
+      <c r="K117" s="2"/>
       <c r="L117" s="2" t="s">
         <v>19</v>
       </c>
@@ -6314,13 +6082,11 @@
       <c r="H118" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I118" s="2"/>
-      <c r="J118" s="3">
+      <c r="I118" s="2">
         <v>317</v>
       </c>
-      <c r="K118" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J118" s="2"/>
+      <c r="K118" s="2"/>
       <c r="L118" s="2" t="s">
         <v>19</v>
       </c>
@@ -6353,13 +6119,11 @@
       <c r="H119" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I119" s="2"/>
-      <c r="J119" s="3">
+      <c r="I119" s="2">
         <v>317</v>
       </c>
-      <c r="K119" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J119" s="2"/>
+      <c r="K119" s="2"/>
       <c r="L119" s="2" t="s">
         <v>19</v>
       </c>
@@ -6394,13 +6158,11 @@
       <c r="H120" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I120" s="2"/>
-      <c r="J120" s="3">
+      <c r="I120" s="2">
         <v>317</v>
       </c>
-      <c r="K120" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J120" s="2"/>
+      <c r="K120" s="2"/>
       <c r="L120" s="2" t="s">
         <v>19</v>
       </c>
@@ -6435,13 +6197,11 @@
       <c r="H121" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I121" s="2"/>
-      <c r="J121" s="3">
+      <c r="I121" s="2">
         <v>201</v>
       </c>
-      <c r="K121" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J121" s="2"/>
+      <c r="K121" s="2"/>
       <c r="L121" s="2" t="s">
         <v>19</v>
       </c>
@@ -6474,13 +6234,11 @@
       <c r="H122" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I122" s="2"/>
-      <c r="J122" s="3">
+      <c r="I122" s="2">
         <v>201</v>
       </c>
-      <c r="K122" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J122" s="2"/>
+      <c r="K122" s="2"/>
       <c r="L122" s="2" t="s">
         <v>19</v>
       </c>
@@ -6513,13 +6271,11 @@
       <c r="H123" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I123" s="2"/>
-      <c r="J123" s="3">
+      <c r="I123" s="2">
         <v>317</v>
       </c>
-      <c r="K123" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J123" s="2"/>
+      <c r="K123" s="2"/>
       <c r="L123" s="2" t="s">
         <v>19</v>
       </c>
@@ -6552,13 +6308,11 @@
       <c r="H124" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I124" s="2"/>
-      <c r="J124" s="3">
+      <c r="I124" s="2">
         <v>317</v>
       </c>
-      <c r="K124" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J124" s="2"/>
+      <c r="K124" s="2"/>
       <c r="L124" s="2" t="s">
         <v>19</v>
       </c>
@@ -6592,10 +6346,8 @@
         <v>37</v>
       </c>
       <c r="I125" s="2"/>
-      <c r="J125" s="3"/>
-      <c r="K125" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J125" s="2"/>
+      <c r="K125" s="2"/>
       <c r="L125" s="2" t="s">
         <v>19</v>
       </c>
@@ -6628,13 +6380,11 @@
       <c r="H126" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I126" s="2"/>
-      <c r="J126" s="3" t="s">
+      <c r="I126" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="K126" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J126" s="2"/>
+      <c r="K126" s="2"/>
       <c r="L126" s="2" t="s">
         <v>19</v>
       </c>
@@ -6667,13 +6417,11 @@
       <c r="H127" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I127" s="2"/>
-      <c r="J127" s="3">
-        <v>37</v>
-      </c>
-      <c r="K127" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="I127" s="2">
+        <v>37</v>
+      </c>
+      <c r="J127" s="2"/>
+      <c r="K127" s="2"/>
       <c r="L127" s="2" t="s">
         <v>19</v>
       </c>
@@ -6706,13 +6454,11 @@
       <c r="H128" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I128" s="2"/>
-      <c r="J128" s="3">
+      <c r="I128" s="2">
         <v>205</v>
       </c>
-      <c r="K128" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J128" s="2"/>
+      <c r="K128" s="2"/>
       <c r="L128" s="2" t="s">
         <v>19</v>
       </c>
@@ -6746,10 +6492,8 @@
         <v>37</v>
       </c>
       <c r="I129" s="2"/>
-      <c r="J129" s="3"/>
-      <c r="K129" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J129" s="2"/>
+      <c r="K129" s="2"/>
       <c r="L129" s="2" t="s">
         <v>19</v>
       </c>
@@ -6783,10 +6527,8 @@
         <v>37</v>
       </c>
       <c r="I130" s="2"/>
-      <c r="J130" s="3"/>
-      <c r="K130" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J130" s="2"/>
+      <c r="K130" s="2"/>
       <c r="L130" s="2" t="s">
         <v>19</v>
       </c>
@@ -6820,10 +6562,8 @@
         <v>37</v>
       </c>
       <c r="I131" s="2"/>
-      <c r="J131" s="3"/>
-      <c r="K131" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J131" s="2"/>
+      <c r="K131" s="2"/>
       <c r="L131" s="2" t="s">
         <v>19</v>
       </c>
@@ -6857,10 +6597,8 @@
         <v>37</v>
       </c>
       <c r="I132" s="2"/>
-      <c r="J132" s="3"/>
-      <c r="K132" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J132" s="2"/>
+      <c r="K132" s="2"/>
       <c r="L132" s="2" t="s">
         <v>19</v>
       </c>
@@ -6894,10 +6632,8 @@
         <v>37</v>
       </c>
       <c r="I133" s="2"/>
-      <c r="J133" s="3"/>
-      <c r="K133" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J133" s="2"/>
+      <c r="K133" s="2"/>
       <c r="L133" s="2" t="s">
         <v>19</v>
       </c>
@@ -6931,10 +6667,8 @@
         <v>37</v>
       </c>
       <c r="I134" s="2"/>
-      <c r="J134" s="3"/>
-      <c r="K134" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J134" s="2"/>
+      <c r="K134" s="2"/>
       <c r="L134" s="2" t="s">
         <v>19</v>
       </c>
@@ -6968,10 +6702,8 @@
         <v>37</v>
       </c>
       <c r="I135" s="2"/>
-      <c r="J135" s="3"/>
-      <c r="K135" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J135" s="2"/>
+      <c r="K135" s="2"/>
       <c r="L135" s="2" t="s">
         <v>19</v>
       </c>
@@ -7007,10 +6739,8 @@
         <v>37</v>
       </c>
       <c r="I136" s="2"/>
-      <c r="J136" s="3"/>
-      <c r="K136" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J136" s="2"/>
+      <c r="K136" s="2"/>
       <c r="L136" s="2" t="s">
         <v>19</v>
       </c>
@@ -7046,10 +6776,8 @@
         <v>37</v>
       </c>
       <c r="I137" s="2"/>
-      <c r="J137" s="3"/>
-      <c r="K137" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J137" s="2"/>
+      <c r="K137" s="2"/>
       <c r="L137" s="2" t="s">
         <v>19</v>
       </c>
@@ -7082,13 +6810,11 @@
       <c r="H138" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I138" s="2"/>
-      <c r="J138" s="3" t="s">
+      <c r="I138" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="K138" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J138" s="2"/>
+      <c r="K138" s="2"/>
       <c r="L138" s="2" t="s">
         <v>19</v>
       </c>
@@ -7124,10 +6850,8 @@
         <v>37</v>
       </c>
       <c r="I139" s="2"/>
-      <c r="J139" s="3"/>
-      <c r="K139" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J139" s="2"/>
+      <c r="K139" s="2"/>
       <c r="L139" s="2" t="s">
         <v>19</v>
       </c>
@@ -7163,10 +6887,8 @@
         <v>37</v>
       </c>
       <c r="I140" s="2"/>
-      <c r="J140" s="3"/>
-      <c r="K140" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J140" s="2"/>
+      <c r="K140" s="2"/>
       <c r="L140" s="2" t="s">
         <v>19</v>
       </c>
@@ -7200,10 +6922,8 @@
         <v>37</v>
       </c>
       <c r="I141" s="2"/>
-      <c r="J141" s="3"/>
-      <c r="K141" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J141" s="2"/>
+      <c r="K141" s="2"/>
       <c r="L141" s="2" t="s">
         <v>19</v>
       </c>
@@ -7237,10 +6957,8 @@
         <v>37</v>
       </c>
       <c r="I142" s="2"/>
-      <c r="J142" s="3"/>
-      <c r="K142" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J142" s="2"/>
+      <c r="K142" s="2"/>
       <c r="L142" s="2" t="s">
         <v>19</v>
       </c>
@@ -7274,10 +6992,8 @@
         <v>37</v>
       </c>
       <c r="I143" s="2"/>
-      <c r="J143" s="3"/>
-      <c r="K143" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J143" s="2"/>
+      <c r="K143" s="2"/>
       <c r="L143" s="2" t="s">
         <v>19</v>
       </c>
@@ -7311,10 +7027,8 @@
         <v>37</v>
       </c>
       <c r="I144" s="2"/>
-      <c r="J144" s="3"/>
-      <c r="K144" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J144" s="2"/>
+      <c r="K144" s="2"/>
       <c r="L144" s="2" t="s">
         <v>19</v>
       </c>
@@ -7348,10 +7062,8 @@
         <v>37</v>
       </c>
       <c r="I145" s="2"/>
-      <c r="J145" s="3"/>
-      <c r="K145" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J145" s="2"/>
+      <c r="K145" s="2"/>
       <c r="L145" s="2" t="s">
         <v>19</v>
       </c>
@@ -7385,10 +7097,8 @@
         <v>37</v>
       </c>
       <c r="I146" s="2"/>
-      <c r="J146" s="3"/>
-      <c r="K146" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J146" s="2"/>
+      <c r="K146" s="2"/>
       <c r="L146" s="2" t="s">
         <v>19</v>
       </c>
@@ -7421,13 +7131,11 @@
       <c r="H147" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I147" s="2"/>
-      <c r="J147" s="3">
+      <c r="I147" s="2">
         <v>28</v>
       </c>
-      <c r="K147" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J147" s="2"/>
+      <c r="K147" s="2"/>
       <c r="L147" s="2" t="s">
         <v>19</v>
       </c>
@@ -7462,13 +7170,11 @@
       <c r="H148" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I148" s="2"/>
-      <c r="J148" s="3">
+      <c r="I148" s="2">
         <v>28</v>
       </c>
-      <c r="K148" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J148" s="2"/>
+      <c r="K148" s="2"/>
       <c r="L148" s="2" t="s">
         <v>19</v>
       </c>
@@ -7502,10 +7208,8 @@
         <v>37</v>
       </c>
       <c r="I149" s="2"/>
-      <c r="J149" s="3"/>
-      <c r="K149" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J149" s="2"/>
+      <c r="K149" s="2"/>
       <c r="L149" s="2" t="s">
         <v>18</v>
       </c>
@@ -7538,15 +7242,13 @@
       <c r="H150" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I150" s="2" t="s">
+      <c r="I150" s="2">
+        <v>111</v>
+      </c>
+      <c r="J150" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="J150" s="3">
-        <v>111</v>
-      </c>
-      <c r="K150" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="K150" s="2"/>
       <c r="L150" s="2" t="s">
         <v>18</v>
       </c>
@@ -7580,10 +7282,8 @@
         <v>37</v>
       </c>
       <c r="I151" s="2"/>
-      <c r="J151" s="3"/>
-      <c r="K151" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J151" s="2"/>
+      <c r="K151" s="2"/>
       <c r="L151" s="2" t="s">
         <v>19</v>
       </c>
@@ -7617,10 +7317,8 @@
         <v>37</v>
       </c>
       <c r="I152" s="2"/>
-      <c r="J152" s="3"/>
-      <c r="K152" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J152" s="2"/>
+      <c r="K152" s="2"/>
       <c r="L152" s="2" t="s">
         <v>19</v>
       </c>
@@ -7654,10 +7352,8 @@
         <v>37</v>
       </c>
       <c r="I153" s="2"/>
-      <c r="J153" s="3"/>
-      <c r="K153" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J153" s="2"/>
+      <c r="K153" s="2"/>
       <c r="L153" s="2" t="s">
         <v>19</v>
       </c>
@@ -7691,10 +7387,8 @@
         <v>37</v>
       </c>
       <c r="I154" s="2"/>
-      <c r="J154" s="3"/>
-      <c r="K154" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J154" s="2"/>
+      <c r="K154" s="2"/>
       <c r="L154" s="2" t="s">
         <v>19</v>
       </c>
@@ -7728,10 +7422,8 @@
         <v>37</v>
       </c>
       <c r="I155" s="2"/>
-      <c r="J155" s="3"/>
-      <c r="K155" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J155" s="2"/>
+      <c r="K155" s="2"/>
       <c r="L155" s="2" t="s">
         <v>19</v>
       </c>
@@ -7765,10 +7457,8 @@
         <v>37</v>
       </c>
       <c r="I156" s="2"/>
-      <c r="J156" s="3"/>
-      <c r="K156" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J156" s="2"/>
+      <c r="K156" s="2"/>
       <c r="L156" s="2" t="s">
         <v>19</v>
       </c>
@@ -7802,10 +7492,8 @@
         <v>37</v>
       </c>
       <c r="I157" s="2"/>
-      <c r="J157" s="3"/>
-      <c r="K157" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J157" s="2"/>
+      <c r="K157" s="2"/>
       <c r="L157" s="2" t="s">
         <v>19</v>
       </c>
@@ -7839,10 +7527,8 @@
         <v>37</v>
       </c>
       <c r="I158" s="2"/>
-      <c r="J158" s="3"/>
-      <c r="K158" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J158" s="2"/>
+      <c r="K158" s="2"/>
       <c r="L158" s="2" t="s">
         <v>19</v>
       </c>
@@ -7876,10 +7562,8 @@
         <v>37</v>
       </c>
       <c r="I159" s="2"/>
-      <c r="J159" s="3"/>
-      <c r="K159" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J159" s="2"/>
+      <c r="K159" s="2"/>
       <c r="L159" s="2" t="s">
         <v>19</v>
       </c>
@@ -7913,10 +7597,8 @@
         <v>37</v>
       </c>
       <c r="I160" s="2"/>
-      <c r="J160" s="3"/>
-      <c r="K160" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J160" s="2"/>
+      <c r="K160" s="2"/>
       <c r="L160" s="2" t="s">
         <v>19</v>
       </c>
@@ -7950,10 +7632,8 @@
         <v>37</v>
       </c>
       <c r="I161" s="2"/>
-      <c r="J161" s="3"/>
-      <c r="K161" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J161" s="2"/>
+      <c r="K161" s="2"/>
       <c r="L161" s="2" t="s">
         <v>19</v>
       </c>
@@ -7987,10 +7667,8 @@
         <v>37</v>
       </c>
       <c r="I162" s="2"/>
-      <c r="J162" s="3"/>
-      <c r="K162" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J162" s="2"/>
+      <c r="K162" s="2"/>
       <c r="L162" s="2" t="s">
         <v>19</v>
       </c>
@@ -8026,10 +7704,8 @@
         <v>37</v>
       </c>
       <c r="I163" s="2"/>
-      <c r="J163" s="3"/>
-      <c r="K163" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J163" s="2"/>
+      <c r="K163" s="2"/>
       <c r="L163" s="2" t="s">
         <v>19</v>
       </c>
@@ -8065,10 +7741,8 @@
         <v>37</v>
       </c>
       <c r="I164" s="2"/>
-      <c r="J164" s="3"/>
-      <c r="K164" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J164" s="2"/>
+      <c r="K164" s="2"/>
       <c r="L164" s="2" t="s">
         <v>19</v>
       </c>
@@ -8102,10 +7776,8 @@
         <v>37</v>
       </c>
       <c r="I165" s="2"/>
-      <c r="J165" s="3"/>
-      <c r="K165" s="2" t="s">
-        <v>19</v>
-      </c>
+      <c r="J165" s="2"/>
+      <c r="K165" s="2"/>
       <c r="L165" s="2" t="s">
         <v>19</v>
       </c>

</xml_diff>